<commit_message>
Actualizacion cuadro mora casi finalizacion
</commit_message>
<xml_diff>
--- a/Edificio Miraflores/reporte_mora_miraflores.xlsx
+++ b/Edificio Miraflores/reporte_mora_miraflores.xlsx
@@ -469,16 +469,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
@@ -493,7 +493,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Departamento 3C - JOSE MANUEL BUSTILLOS</t>
+          <t>Departamento 3E - JULIETA MAMANI DE NINA</t>
         </is>
       </c>
     </row>
@@ -505,20 +505,85 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>jun-25</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>jul-25</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ago-25</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>sep-25</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>oct-25</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>nov-25</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>dic-25</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>ene-26</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>feb-26</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
           <t>jul-26</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>ago-26</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -531,23 +596,62 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>157.48</v>
+        <v>209</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>163.53</v>
+        <v>217</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>163.02</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>484.03</v>
+        <v>220.05</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>201.11</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>220.27</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>219.73</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>212.42</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>217</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>258.4</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>258.02</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>271.94</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>255.3</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>280.97</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>268.06</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>238.98</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>237.66</v>
+      </c>
+      <c r="R3" s="5" t="n">
+        <v>3785.91</v>
       </c>
     </row>
     <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Departamento 3E - JULIETA MAMANI DE NINA</t>
+          <t>Departamento 22B - FABIOLA LAURA VARGAS</t>
         </is>
       </c>
     </row>
@@ -559,85 +663,60 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>jun-25</t>
+          <t>nov-25</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>jul-25</t>
+          <t>dic-25</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ago-25</t>
+          <t>ene-26</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>sep-25</t>
+          <t>feb-26</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>oct-25</t>
+          <t>mar-26</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>nov-25</t>
+          <t>abr-26</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>dic-25</t>
+          <t>may-26</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>ene-26</t>
+          <t>jun-26</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>feb-26</t>
+          <t>jul-26</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>mar-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>abr-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -650,62 +729,47 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>209</v>
+        <v>292.3</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>217</v>
+        <v>263.15</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>220.05</v>
+        <v>282.93</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>201.11</v>
+        <v>317.65</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>220.27</v>
+        <v>317.78</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>219.73</v>
+        <v>336.63</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>212.42</v>
+        <v>317</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>217</v>
+        <v>317</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>258.4</v>
+        <v>317</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>258.02</v>
+        <v>317</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>271.94</v>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>255.3</v>
-      </c>
-      <c r="N7" s="4" t="n">
-        <v>280.97</v>
-      </c>
-      <c r="O7" s="4" t="n">
-        <v>268.06</v>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>238.98</v>
-      </c>
-      <c r="Q7" s="4" t="n">
-        <v>237.66</v>
-      </c>
-      <c r="R7" s="5" t="n">
-        <v>3785.91</v>
+        <v>342.22</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>3420.66</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Departamento 4B - MANUEL A. LIRA ORTIZ</t>
+          <t>Departamento 9B - PEDRO CALANI/ANA C. DONAIRE</t>
         </is>
       </c>
     </row>
@@ -717,45 +781,25 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>feb-26</t>
+          <t>gestiones anteriores</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>mar-26</t>
+          <t>oct-25</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>abr-26</t>
+          <t>nov-25</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>may-26</t>
+          <t>dic-25</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -768,38 +812,26 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>194.31</v>
+        <v>2175</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>162.49</v>
+        <v>168.07</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>167.19</v>
+        <v>170.59</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>167.19</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>191.31</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>196.17</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>190.87</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>183.74</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>1453.27</v>
+        <v>165</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>2678.66</v>
       </c>
     </row>
     <row r="12"/>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Departamento 4C - SIRLEY VALENCIA/ANGEL VALENCVIA SIRPA</t>
+          <t>Departamento 13C - IVAN ORLANDO MIRANDA TICONA</t>
         </is>
       </c>
     </row>
@@ -811,10 +843,70 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>sep-25</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>oct-25</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>nov-25</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>dic-25</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>ene-26</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>feb-26</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -827,17 +919,53 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>173.45</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>173.45</v>
+        <v>152.71</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>152.29</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>152.38</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>152.84</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>152.5</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>190.49</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>188.45</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>188.42</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>203.07</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>213.82</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>205.76</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>207.26</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>207.59</v>
+      </c>
+      <c r="O15" s="5" t="n">
+        <v>2367.58</v>
       </c>
     </row>
     <row r="16"/>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Departamento 4E - ELIZABETH PAREDES SARDON</t>
+          <t>Departamento 18C - SANDRA MALLEA</t>
         </is>
       </c>
     </row>
@@ -849,10 +977,90 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>may-25</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>jun-25</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>jul-25</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>ago-25</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>sep-25</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>oct-25</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>nov-25</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>dic-25</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>ene-26</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>feb-26</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -865,17 +1073,65 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>342.24</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>342.24</v>
+        <v>116</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>114.11</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>114.08</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>114.17</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>114.21</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>114</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>114</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>145.3</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>145.04</v>
+      </c>
+      <c r="M19" s="4" t="n">
+        <v>145.37</v>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>145.46</v>
+      </c>
+      <c r="O19" s="4" t="n">
+        <v>145.23</v>
+      </c>
+      <c r="P19" s="4" t="n">
+        <v>145.29</v>
+      </c>
+      <c r="Q19" s="4" t="n">
+        <v>145.33</v>
+      </c>
+      <c r="R19" s="4" t="n">
+        <v>146.57</v>
+      </c>
+      <c r="S19" s="5" t="n">
+        <v>2196.16</v>
       </c>
     </row>
     <row r="20"/>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Departamento 4F - LOURDES LIMA TELLEZ</t>
+          <t>Departamento 12B - PABLO FERNANDEZ B/JOEL HERNANDEZ</t>
         </is>
       </c>
     </row>
@@ -887,10 +1143,50 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>ene-26</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>feb-26</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -903,17 +1199,41 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>185.45</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>185.45</v>
+        <v>203.6</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>275.35</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>251.59</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>237.2</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>261.75</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>250.74</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>211.53</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>226.89</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>255.51</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>2174.16</v>
       </c>
     </row>
     <row r="24"/>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>Departamento 5A - MAIDA MENDIA/ JAIME TAKATA</t>
+          <t>Departamento 10D - DIEGO QUINTEROS SAAVEDRA</t>
         </is>
       </c>
     </row>
@@ -925,15 +1245,50 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
+          <t>ges_ant</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>feb-26</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
           <t>ago-26</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -946,20 +1301,41 @@
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>225.01</v>
+        <v>384</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>219.61</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>444.62</v>
+        <v>146.16</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>153.28</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>151.58</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>155.03</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>153.52</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>158.86</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>165.29</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>155.25</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>1622.97</v>
       </c>
     </row>
     <row r="28"/>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>Departamento 5B - CINTIA ALVARADO/SAMUEL LIMACHI</t>
+          <t>Departamento 4B - MANUEL A. LIRA ORTIZ</t>
         </is>
       </c>
     </row>
@@ -971,25 +1347,45 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>feb-26</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
           <t>jun-26</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>jul-26</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>ago-26</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1002,26 +1398,38 @@
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>261.71</v>
+        <v>194.31</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>243.33</v>
+        <v>162.49</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>226.72</v>
+        <v>167.19</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>208.25</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>940.01</v>
+        <v>167.19</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>191.31</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>196.17</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>190.87</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>183.74</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>1453.27</v>
       </c>
     </row>
     <row r="32"/>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>Departamento 5C - LUZ  TICONA QUISPE</t>
+          <t>Departamento 15E - WILMA IGLESIAS BEDOYA</t>
         </is>
       </c>
     </row>
@@ -1033,10 +1441,95 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>abr-25</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>may-25</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>jun-25</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>jul-25</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>ago-25</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>sep-25</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>oct-25</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>nov-25</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>dic-25</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>ene-26</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>feb-26</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1049,17 +1542,68 @@
         </is>
       </c>
       <c r="B35" s="4" t="n">
-        <v>179.21</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>179.21</v>
+        <v>37</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>36.71</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>36.98</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>186.21</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>36.38</v>
+      </c>
+      <c r="L35" s="4" t="n">
+        <v>86.25</v>
+      </c>
+      <c r="M35" s="4" t="n">
+        <v>94.01000000000001</v>
+      </c>
+      <c r="N35" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="O35" s="4" t="n">
+        <v>90.37</v>
+      </c>
+      <c r="P35" s="4" t="n">
+        <v>89.88</v>
+      </c>
+      <c r="Q35" s="4" t="n">
+        <v>50.91</v>
+      </c>
+      <c r="R35" s="4" t="n">
+        <v>241.35</v>
+      </c>
+      <c r="S35" s="4" t="n">
+        <v>242.02</v>
+      </c>
+      <c r="T35" s="5" t="n">
+        <v>1430.78</v>
       </c>
     </row>
     <row r="36"/>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>Departamento 5D - MARCELO LOZA/ MARCOS RODRIGUEZ</t>
+          <t>Departamento 6B - PALMIRA ARANDIA DE CALDERON/BORIS C</t>
         </is>
       </c>
     </row>
@@ -1071,10 +1615,30 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>may-26</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1087,17 +1651,29 @@
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>125.2</v>
-      </c>
-      <c r="C39" s="5" t="n">
-        <v>125.2</v>
+        <v>238.44</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>248.59</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>243.11</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>256.01</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>256.83</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>1242.98</v>
       </c>
     </row>
     <row r="40"/>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>Departamento 5E - GERMAN HUANCA C./EMILIANA MAMANI</t>
+          <t>Departamento 13F - HUGO MACHICADO</t>
         </is>
       </c>
     </row>
@@ -1109,45 +1685,35 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>feb-26</t>
+          <t>abr-26</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>mar-26</t>
+          <t>may-26</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>abr-26</t>
+          <t>jun-26</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>may-26</t>
+          <t>jul-26</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>jun-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>jul-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1160,38 +1726,32 @@
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>50</v>
+        <v>171.68</v>
       </c>
       <c r="C43" s="4" t="n">
-        <v>40</v>
+        <v>177.96</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>40</v>
+        <v>173.05</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>40</v>
+        <v>170.83</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>50</v>
+        <v>180.15</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>49.94</v>
-      </c>
-      <c r="H43" s="4" t="n">
-        <v>52.39</v>
-      </c>
-      <c r="I43" s="4" t="n">
-        <v>240.85</v>
-      </c>
-      <c r="J43" s="5" t="n">
-        <v>563.1800000000001</v>
+        <v>177.59</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>1051.26</v>
       </c>
     </row>
     <row r="44"/>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>Departamento 5F - ROCIO MABEL ALBERTO PATY</t>
+          <t>Departamento 5B - CINTIA ALVARADO/SAMUEL LIMACHI</t>
         </is>
       </c>
     </row>
@@ -1203,10 +1763,25 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>jun-26</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1219,17 +1794,26 @@
         </is>
       </c>
       <c r="B47" s="4" t="n">
-        <v>203.81</v>
-      </c>
-      <c r="C47" s="5" t="n">
-        <v>203.81</v>
+        <v>261.71</v>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>243.33</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>226.72</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>208.25</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>940.01</v>
       </c>
     </row>
     <row r="48"/>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>Departamento 6B - PALMIRA ARANDIA DE CALDERON/BORIS C</t>
+          <t>Departamento 12E - BLANCA MIRANDA/LUIGUI VARGAS</t>
         </is>
       </c>
     </row>
@@ -1241,30 +1825,45 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
+          <t>feb-26</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
           <t>may-26</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>jun-26</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>jul-26</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>ago-26</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1277,29 +1876,38 @@
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>238.44</v>
+        <v>54</v>
       </c>
       <c r="C51" s="4" t="n">
-        <v>248.59</v>
+        <v>54</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>243.11</v>
+        <v>54</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>256.01</v>
+        <v>54</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>256.83</v>
-      </c>
-      <c r="G51" s="5" t="n">
-        <v>1242.98</v>
+        <v>54</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>335.97</v>
+      </c>
+      <c r="J51" s="5" t="n">
+        <v>709.97</v>
       </c>
     </row>
     <row r="52"/>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>Departamento 6E - PAULINA CRUZ PINTO</t>
+          <t>Departamento 14E - CIDAL LTDA</t>
         </is>
       </c>
     </row>
@@ -1311,30 +1919,20 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>may-26</t>
+          <t>jul-26</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>jun-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>jul-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1347,29 +1945,23 @@
         </is>
       </c>
       <c r="B55" s="4" t="n">
-        <v>50</v>
+        <v>236</v>
       </c>
       <c r="C55" s="4" t="n">
-        <v>50</v>
+        <v>236</v>
       </c>
       <c r="D55" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="E55" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F55" s="4" t="n">
-        <v>265.38</v>
-      </c>
-      <c r="G55" s="5" t="n">
-        <v>465.38</v>
+        <v>236.39</v>
+      </c>
+      <c r="E55" s="5" t="n">
+        <v>708.39</v>
       </c>
     </row>
     <row r="56"/>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>Departamento 6F - BEATRIZ GONZALES DURAN</t>
+          <t>Departamento 20B - RAQUEL GUTIERREZ FLORES</t>
         </is>
       </c>
     </row>
@@ -1381,10 +1973,20 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>jul-26</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1397,17 +1999,23 @@
         </is>
       </c>
       <c r="B59" s="4" t="n">
-        <v>212.31</v>
-      </c>
-      <c r="C59" s="5" t="n">
-        <v>212.31</v>
+        <v>228.7</v>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>231.79</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>226.48</v>
+      </c>
+      <c r="E59" s="5" t="n">
+        <v>686.97</v>
       </c>
     </row>
     <row r="60"/>
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>Departamento 7A - EDUARDO FERNANDEZ</t>
+          <t>Departamento 10B - JOSE LUIS QUISPE FLORES</t>
         </is>
       </c>
     </row>
@@ -1419,10 +2027,25 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>jun-26</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1435,17 +2058,26 @@
         </is>
       </c>
       <c r="B63" s="4" t="n">
-        <v>211.42</v>
-      </c>
-      <c r="C63" s="5" t="n">
-        <v>211.42</v>
+        <v>162</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="F63" s="5" t="n">
+        <v>648</v>
       </c>
     </row>
     <row r="64"/>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>Departamento 7D - MARTHA LIZARAZU/FROILAN LOPEZ CH.</t>
+          <t>Departamento 5E - GERMAN HUANCA C./EMILIANA MAMANI</t>
         </is>
       </c>
     </row>
@@ -1457,10 +2089,45 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>feb-26</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1473,17 +2140,38 @@
         </is>
       </c>
       <c r="B67" s="4" t="n">
-        <v>92.09999999999999</v>
-      </c>
-      <c r="C67" s="5" t="n">
-        <v>92.09999999999999</v>
+        <v>50</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>52.39</v>
+      </c>
+      <c r="I67" s="4" t="n">
+        <v>240.85</v>
+      </c>
+      <c r="J67" s="5" t="n">
+        <v>563.1800000000001</v>
       </c>
     </row>
     <row r="68"/>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>Departamento 7F - ROMAN CALDERON/ANGELA TERRAZAS M.</t>
+          <t>Departamento 20DE - GRACE FERNANDEZ</t>
         </is>
       </c>
     </row>
@@ -1495,10 +2183,45 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>feb-26</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>mar-26</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>abr-26</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>may-26</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1511,17 +2234,38 @@
         </is>
       </c>
       <c r="B71" s="4" t="n">
-        <v>168.73</v>
-      </c>
-      <c r="C71" s="5" t="n">
-        <v>168.73</v>
+        <v>70</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>70.03</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>69.97</v>
+      </c>
+      <c r="H71" s="4" t="n">
+        <v>69.97</v>
+      </c>
+      <c r="I71" s="4" t="n">
+        <v>69.95999999999999</v>
+      </c>
+      <c r="J71" s="5" t="n">
+        <v>559.9300000000001</v>
       </c>
     </row>
     <row r="72"/>
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>Departamento 8A -  MOISES CABRERA/ELIANA TORRES</t>
+          <t>Departamento 16A - PABEL SAINZ E,/ERICK JARANDILLA</t>
         </is>
       </c>
     </row>
@@ -1533,10 +2277,20 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
           <t>ago-26</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1549,17 +2303,23 @@
         </is>
       </c>
       <c r="B75" s="4" t="n">
-        <v>253.48</v>
-      </c>
-      <c r="C75" s="5" t="n">
-        <v>253.48</v>
+        <v>180.63</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>177.85</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>173.14</v>
+      </c>
+      <c r="E75" s="5" t="n">
+        <v>531.62</v>
       </c>
     </row>
     <row r="76"/>
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>Departamento 8C - CARLOS ALIAGA LIMA</t>
+          <t>Departamento 3C - JOSE MANUEL BUSTILLOS</t>
         </is>
       </c>
     </row>
@@ -1571,10 +2331,20 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>jul-26</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1587,17 +2357,23 @@
         </is>
       </c>
       <c r="B79" s="4" t="n">
-        <v>188.46</v>
-      </c>
-      <c r="C79" s="5" t="n">
-        <v>188.46</v>
+        <v>157.48</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>163.53</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>163.02</v>
+      </c>
+      <c r="E79" s="5" t="n">
+        <v>484.03</v>
       </c>
     </row>
     <row r="80"/>
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>Departamento 8E - WARA SALINAS NINA</t>
+          <t>Departamento 6E - PAULINA CRUZ PINTO</t>
         </is>
       </c>
     </row>
@@ -1609,10 +2385,30 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>may-26</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1625,17 +2421,29 @@
         </is>
       </c>
       <c r="B83" s="4" t="n">
-        <v>243.05</v>
-      </c>
-      <c r="C83" s="5" t="n">
-        <v>243.05</v>
+        <v>50</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>265.38</v>
+      </c>
+      <c r="G83" s="5" t="n">
+        <v>465.38</v>
       </c>
     </row>
     <row r="84"/>
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>Departamento 9B - PEDRO CALANI/ANA C. DONAIRE</t>
+          <t>Departamento 14D - JAVIER RODRIGO OJEDA OICAMPO</t>
         </is>
       </c>
     </row>
@@ -1647,25 +2455,20 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>oct-25</t>
+          <t>jul-26</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>nov-25</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>dic-25</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>ges_ant</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1678,26 +2481,23 @@
         </is>
       </c>
       <c r="B87" s="4" t="n">
-        <v>168.07</v>
+        <v>151.85</v>
       </c>
       <c r="C87" s="4" t="n">
-        <v>170.59</v>
+        <v>152.36</v>
       </c>
       <c r="D87" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="E87" s="4" t="n">
-        <v>2175</v>
-      </c>
-      <c r="F87" s="5" t="n">
-        <v>2678.66</v>
+        <v>148.59</v>
+      </c>
+      <c r="E87" s="5" t="n">
+        <v>452.8000000000001</v>
       </c>
     </row>
     <row r="88"/>
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>Departamento 10A - MARCELO USCAMAITA</t>
+          <t>Departamento 5A - MAIDA MENDIA/ JAIME TAKATA</t>
         </is>
       </c>
     </row>
@@ -1709,10 +2509,15 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1725,17 +2530,20 @@
         </is>
       </c>
       <c r="B91" s="4" t="n">
-        <v>166.29</v>
-      </c>
-      <c r="C91" s="5" t="n">
-        <v>166.29</v>
+        <v>225.01</v>
+      </c>
+      <c r="C91" s="4" t="n">
+        <v>219.61</v>
+      </c>
+      <c r="D91" s="5" t="n">
+        <v>444.62</v>
       </c>
     </row>
     <row r="92"/>
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>Departamento 10B - JOSE LUIS QUISPE FLORES</t>
+          <t>Departamento 11C - ANA A. URIA PONCE/ JORGE VASQUEZ</t>
         </is>
       </c>
     </row>
@@ -1747,25 +2555,15 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>jun-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>jul-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1778,26 +2576,20 @@
         </is>
       </c>
       <c r="B95" s="4" t="n">
-        <v>162</v>
+        <v>213.38</v>
       </c>
       <c r="C95" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="D95" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="E95" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="F95" s="5" t="n">
-        <v>648</v>
+        <v>212.52</v>
+      </c>
+      <c r="D95" s="5" t="n">
+        <v>425.9</v>
       </c>
     </row>
     <row r="96"/>
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>Departamento 10D - DIEGO QUINTEROS SAAVEDRA</t>
+          <t>Departamento 13A - CLAUDIA COAQUIRA AYAVIRI</t>
         </is>
       </c>
     </row>
@@ -1809,50 +2601,15 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>feb-26</t>
+          <t>mar-26</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>mar-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>abr-26</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="G98" s="2" t="inlineStr">
-        <is>
-          <t>ges_ant</t>
-        </is>
-      </c>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="I98" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="J98" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="K98" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1865,34 +2622,13 @@
         </is>
       </c>
       <c r="B99" s="4" t="n">
-        <v>146.16</v>
+        <v>192.27</v>
       </c>
       <c r="C99" s="4" t="n">
-        <v>153.28</v>
-      </c>
-      <c r="D99" s="4" t="n">
-        <v>151.58</v>
-      </c>
-      <c r="E99" s="4" t="n">
-        <v>155.03</v>
-      </c>
-      <c r="F99" s="4" t="n">
-        <v>153.52</v>
-      </c>
-      <c r="G99" s="4" t="n">
-        <v>384</v>
-      </c>
-      <c r="H99" s="4" t="n">
-        <v>158.86</v>
-      </c>
-      <c r="I99" s="4" t="n">
-        <v>165.29</v>
-      </c>
-      <c r="J99" s="4" t="n">
-        <v>155.25</v>
-      </c>
-      <c r="K99" s="5" t="n">
-        <v>1622.97</v>
+        <v>200.42</v>
+      </c>
+      <c r="D99" s="5" t="n">
+        <v>392.69</v>
       </c>
     </row>
     <row r="100"/>
@@ -1937,7 +2673,7 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>Departamento 10F - DANIEL GONZALES CUSICANQUI</t>
+          <t xml:space="preserve">Departamento 14C - OSCAR GAUSS CARVAJAL </t>
         </is>
       </c>
     </row>
@@ -1949,10 +2685,15 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1965,17 +2706,20 @@
         </is>
       </c>
       <c r="B107" s="4" t="n">
-        <v>191.93</v>
-      </c>
-      <c r="C107" s="5" t="n">
-        <v>191.93</v>
+        <v>181.01</v>
+      </c>
+      <c r="C107" s="4" t="n">
+        <v>171.39</v>
+      </c>
+      <c r="D107" s="5" t="n">
+        <v>352.4</v>
       </c>
     </row>
     <row r="108"/>
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>Departamento 11B - XIMENA ORELLANA B/</t>
+          <t>Departamento 15F - MICAELA DAFNE ALANES CUBA</t>
         </is>
       </c>
     </row>
@@ -1987,10 +2731,15 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2003,17 +2752,20 @@
         </is>
       </c>
       <c r="B111" s="4" t="n">
-        <v>224.09</v>
-      </c>
-      <c r="C111" s="5" t="n">
-        <v>224.09</v>
+        <v>173.94</v>
+      </c>
+      <c r="C111" s="4" t="n">
+        <v>173.04</v>
+      </c>
+      <c r="D111" s="5" t="n">
+        <v>346.98</v>
       </c>
     </row>
     <row r="112"/>
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>Departamento 11C - ANA A. URIA PONCE/ JORGE VASQUEZ</t>
+          <t>Departamento 4E - ELIZABETH PAREDES SARDON</t>
         </is>
       </c>
     </row>
@@ -2025,15 +2777,10 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>ago-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2046,20 +2793,17 @@
         </is>
       </c>
       <c r="B115" s="4" t="n">
-        <v>213.38</v>
-      </c>
-      <c r="C115" s="4" t="n">
-        <v>212.52</v>
-      </c>
-      <c r="D115" s="5" t="n">
-        <v>425.9</v>
+        <v>342.24</v>
+      </c>
+      <c r="C115" s="5" t="n">
+        <v>342.24</v>
       </c>
     </row>
     <row r="116"/>
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>Departamento 11D - LAURA GEMIO/WILMER CABRERA G.</t>
+          <t>Departamento 18DE - SANDRO MEDRANO</t>
         </is>
       </c>
     </row>
@@ -2071,10 +2815,30 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>may-26</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>jun-26</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>jul-26</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>ago-26</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2087,17 +2851,29 @@
         </is>
       </c>
       <c r="B119" s="4" t="n">
-        <v>132.18</v>
-      </c>
-      <c r="C119" s="5" t="n">
-        <v>132.18</v>
+        <v>69</v>
+      </c>
+      <c r="C119" s="4" t="n">
+        <v>38.66</v>
+      </c>
+      <c r="D119" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="E119" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="F119" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="G119" s="5" t="n">
+        <v>314.66</v>
       </c>
     </row>
     <row r="120"/>
     <row r="121" ht="22" customHeight="1">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>Departamento 12B - PABLO FERNANDEZ B/JOEL HERNANDEZ</t>
+          <t>Departamento 8A -  MOISES CABRERA/ELIANA TORRES</t>
         </is>
       </c>
     </row>
@@ -2109,50 +2885,10 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>ene-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>feb-26</t>
-        </is>
-      </c>
-      <c r="D122" s="2" t="inlineStr">
-        <is>
-          <t>mar-26</t>
-        </is>
-      </c>
-      <c r="E122" s="2" t="inlineStr">
-        <is>
-          <t>abr-26</t>
-        </is>
-      </c>
-      <c r="F122" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="G122" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="H122" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="I122" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="J122" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="K122" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2165,41 +2901,17 @@
         </is>
       </c>
       <c r="B123" s="4" t="n">
-        <v>203.6</v>
-      </c>
-      <c r="C123" s="4" t="n">
-        <v>275.35</v>
-      </c>
-      <c r="D123" s="4" t="n">
-        <v>251.59</v>
-      </c>
-      <c r="E123" s="4" t="n">
-        <v>237.2</v>
-      </c>
-      <c r="F123" s="4" t="n">
-        <v>261.75</v>
-      </c>
-      <c r="G123" s="4" t="n">
-        <v>250.74</v>
-      </c>
-      <c r="H123" s="4" t="n">
-        <v>211.53</v>
-      </c>
-      <c r="I123" s="4" t="n">
-        <v>226.89</v>
-      </c>
-      <c r="J123" s="4" t="n">
-        <v>255.51</v>
-      </c>
-      <c r="K123" s="5" t="n">
-        <v>2174.16</v>
+        <v>253.48</v>
+      </c>
+      <c r="C123" s="5" t="n">
+        <v>253.48</v>
       </c>
     </row>
     <row r="124"/>
     <row r="125" ht="22" customHeight="1">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>Departamento 12C - LISSET MENDEZ/LUIS FERNANDEZ</t>
+          <t>Departamento 8E - WARA SALINAS NINA</t>
         </is>
       </c>
     </row>
@@ -2227,17 +2939,17 @@
         </is>
       </c>
       <c r="B127" s="4" t="n">
-        <v>201.14</v>
+        <v>243.05</v>
       </c>
       <c r="C127" s="5" t="n">
-        <v>201.14</v>
+        <v>243.05</v>
       </c>
     </row>
     <row r="128"/>
     <row r="129" ht="22" customHeight="1">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>Departamento 12D - ERIKA LEON HERBAS</t>
+          <t>Departamento 14B - VANIA ARAOZ PEREZ</t>
         </is>
       </c>
     </row>
@@ -2265,17 +2977,17 @@
         </is>
       </c>
       <c r="B131" s="4" t="n">
-        <v>106.54</v>
+        <v>242.1</v>
       </c>
       <c r="C131" s="5" t="n">
-        <v>106.54</v>
+        <v>242.1</v>
       </c>
     </row>
     <row r="132"/>
     <row r="133" ht="22" customHeight="1">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>Departamento 12E - BLANCA MIRANDA/LUIGUI VARGAS</t>
+          <t>Departamento 11B - XIMENA ORELLANA B/</t>
         </is>
       </c>
     </row>
@@ -2287,45 +2999,10 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>feb-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
-        <is>
-          <t>mar-26</t>
-        </is>
-      </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t>abr-26</t>
-        </is>
-      </c>
-      <c r="E134" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="F134" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="G134" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="H134" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="I134" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="J134" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2338,38 +3015,17 @@
         </is>
       </c>
       <c r="B135" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="C135" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="D135" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="E135" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="F135" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="G135" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="H135" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I135" s="4" t="n">
-        <v>335.97</v>
-      </c>
-      <c r="J135" s="5" t="n">
-        <v>709.97</v>
+        <v>224.09</v>
+      </c>
+      <c r="C135" s="5" t="n">
+        <v>224.09</v>
       </c>
     </row>
     <row r="136"/>
     <row r="137" ht="22" customHeight="1">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>Departamento 13A - CLAUDIA COAQUIRA AYAVIRI</t>
+          <t>Departamento 6F - BEATRIZ GONZALES DURAN</t>
         </is>
       </c>
     </row>
@@ -2381,15 +3037,10 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>mar-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2402,20 +3053,17 @@
         </is>
       </c>
       <c r="B139" s="4" t="n">
-        <v>192.27</v>
-      </c>
-      <c r="C139" s="4" t="n">
-        <v>200.42</v>
-      </c>
-      <c r="D139" s="5" t="n">
-        <v>392.69</v>
+        <v>212.31</v>
+      </c>
+      <c r="C139" s="5" t="n">
+        <v>212.31</v>
       </c>
     </row>
     <row r="140"/>
     <row r="141" ht="22" customHeight="1">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>Departamento 13C - IVAN ORLANDO MIRANDA TICONA</t>
+          <t>Departamento 7A - EDUARDO FERNANDEZ</t>
         </is>
       </c>
     </row>
@@ -2427,70 +3075,10 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>sep-25</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>oct-25</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>nov-25</t>
-        </is>
-      </c>
-      <c r="E142" s="2" t="inlineStr">
-        <is>
-          <t>dic-25</t>
-        </is>
-      </c>
-      <c r="F142" s="2" t="inlineStr">
-        <is>
-          <t>ene-26</t>
-        </is>
-      </c>
-      <c r="G142" s="2" t="inlineStr">
-        <is>
-          <t>feb-26</t>
-        </is>
-      </c>
-      <c r="H142" s="2" t="inlineStr">
-        <is>
-          <t>mar-26</t>
-        </is>
-      </c>
-      <c r="I142" s="2" t="inlineStr">
-        <is>
-          <t>abr-26</t>
-        </is>
-      </c>
-      <c r="J142" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="K142" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="L142" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="M142" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="N142" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="O142" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2503,53 +3091,17 @@
         </is>
       </c>
       <c r="B143" s="4" t="n">
-        <v>152.71</v>
-      </c>
-      <c r="C143" s="4" t="n">
-        <v>152.29</v>
-      </c>
-      <c r="D143" s="4" t="n">
-        <v>152.38</v>
-      </c>
-      <c r="E143" s="4" t="n">
-        <v>152.84</v>
-      </c>
-      <c r="F143" s="4" t="n">
-        <v>152.5</v>
-      </c>
-      <c r="G143" s="4" t="n">
-        <v>190.49</v>
-      </c>
-      <c r="H143" s="4" t="n">
-        <v>188.45</v>
-      </c>
-      <c r="I143" s="4" t="n">
-        <v>188.42</v>
-      </c>
-      <c r="J143" s="4" t="n">
-        <v>203.07</v>
-      </c>
-      <c r="K143" s="4" t="n">
-        <v>213.82</v>
-      </c>
-      <c r="L143" s="4" t="n">
-        <v>205.76</v>
-      </c>
-      <c r="M143" s="4" t="n">
-        <v>207.26</v>
-      </c>
-      <c r="N143" s="4" t="n">
-        <v>207.59</v>
-      </c>
-      <c r="O143" s="5" t="n">
-        <v>2367.58</v>
+        <v>211.42</v>
+      </c>
+      <c r="C143" s="5" t="n">
+        <v>211.42</v>
       </c>
     </row>
     <row r="144"/>
     <row r="145" ht="22" customHeight="1">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>Departamento 13D - MARIA LUISA PEÑALOZA VILA</t>
+          <t>Departamento 5F - ROCIO MABEL ALBERTO PATY</t>
         </is>
       </c>
     </row>
@@ -2561,15 +3113,10 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>ago-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="D146" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2582,20 +3129,17 @@
         </is>
       </c>
       <c r="B147" s="4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C147" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D147" s="5" t="n">
-        <v>0.06</v>
+        <v>203.81</v>
+      </c>
+      <c r="C147" s="5" t="n">
+        <v>203.81</v>
       </c>
     </row>
     <row r="148"/>
     <row r="149" ht="22" customHeight="1">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>Departamento 13F - HUGO MACHICADO</t>
+          <t>Departamento 12C - LISSET MENDEZ/LUIS FERNANDEZ</t>
         </is>
       </c>
     </row>
@@ -2607,35 +3151,10 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>abr-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="E150" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="F150" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="G150" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="H150" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2648,32 +3167,17 @@
         </is>
       </c>
       <c r="B151" s="4" t="n">
-        <v>171.68</v>
-      </c>
-      <c r="C151" s="4" t="n">
-        <v>177.96</v>
-      </c>
-      <c r="D151" s="4" t="n">
-        <v>173.05</v>
-      </c>
-      <c r="E151" s="4" t="n">
-        <v>170.83</v>
-      </c>
-      <c r="F151" s="4" t="n">
-        <v>180.15</v>
-      </c>
-      <c r="G151" s="4" t="n">
-        <v>177.59</v>
-      </c>
-      <c r="H151" s="5" t="n">
-        <v>1051.26</v>
+        <v>201.14</v>
+      </c>
+      <c r="C151" s="5" t="n">
+        <v>201.14</v>
       </c>
     </row>
     <row r="152"/>
     <row r="153" ht="22" customHeight="1">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>Departamento 14B - VANIA ARAOZ PEREZ</t>
+          <t>Departamento 16F - ALVARO ANTICALLE</t>
         </is>
       </c>
     </row>
@@ -2701,17 +3205,17 @@
         </is>
       </c>
       <c r="B155" s="4" t="n">
-        <v>242.1</v>
+        <v>192.48</v>
       </c>
       <c r="C155" s="5" t="n">
-        <v>242.1</v>
+        <v>192.48</v>
       </c>
     </row>
     <row r="156"/>
     <row r="157" ht="22" customHeight="1">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Departamento 14C - OSCAR GAUSS CARVAJAL </t>
+          <t>Departamento 10F - DANIEL GONZALES CUSICANQUI</t>
         </is>
       </c>
     </row>
@@ -2723,15 +3227,10 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>ago-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="D158" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2744,20 +3243,17 @@
         </is>
       </c>
       <c r="B159" s="4" t="n">
-        <v>181.01</v>
-      </c>
-      <c r="C159" s="4" t="n">
-        <v>171.39</v>
-      </c>
-      <c r="D159" s="5" t="n">
-        <v>352.4</v>
+        <v>191.93</v>
+      </c>
+      <c r="C159" s="5" t="n">
+        <v>191.93</v>
       </c>
     </row>
     <row r="160"/>
     <row r="161" ht="22" customHeight="1">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>Departamento 14D - JAVIER RODRIGO OJEDA OICAMPO</t>
+          <t>Departamento 8C - CARLOS ALIAGA LIMA</t>
         </is>
       </c>
     </row>
@@ -2769,20 +3265,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>jul-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="D162" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2795,23 +3281,17 @@
         </is>
       </c>
       <c r="B163" s="4" t="n">
-        <v>151.85</v>
-      </c>
-      <c r="C163" s="4" t="n">
-        <v>152.36</v>
-      </c>
-      <c r="D163" s="4" t="n">
-        <v>148.59</v>
-      </c>
-      <c r="E163" s="5" t="n">
-        <v>452.8000000000001</v>
+        <v>188.46</v>
+      </c>
+      <c r="C163" s="5" t="n">
+        <v>188.46</v>
       </c>
     </row>
     <row r="164"/>
     <row r="165" ht="22" customHeight="1">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>Departamento 14E - CIDAL LTDA</t>
+          <t>Departamento 15C - NANCY CHOQUE/DANIEL RODRIGO M,</t>
         </is>
       </c>
     </row>
@@ -2823,20 +3303,10 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>jul-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="E166" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2849,16 +3319,10 @@
         </is>
       </c>
       <c r="B167" s="4" t="n">
-        <v>236</v>
-      </c>
-      <c r="C167" s="4" t="n">
-        <v>236</v>
-      </c>
-      <c r="D167" s="4" t="n">
-        <v>236.39</v>
-      </c>
-      <c r="E167" s="5" t="n">
-        <v>708.39</v>
+        <v>186.57</v>
+      </c>
+      <c r="C167" s="5" t="n">
+        <v>186.57</v>
       </c>
     </row>
     <row r="168"/>
@@ -2903,7 +3367,7 @@
     <row r="173" ht="22" customHeight="1">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>Departamento 15B - MANUEL RAFAEL HIDALGO/STEFANY RAFAEL</t>
+          <t>Departamento 4F - LOURDES LIMA TELLEZ</t>
         </is>
       </c>
     </row>
@@ -2931,17 +3395,17 @@
         </is>
       </c>
       <c r="B175" s="4" t="n">
-        <v>178.6</v>
+        <v>185.45</v>
       </c>
       <c r="C175" s="5" t="n">
-        <v>178.6</v>
+        <v>185.45</v>
       </c>
     </row>
     <row r="176"/>
     <row r="177" ht="22" customHeight="1">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>Departamento 15C - NANCY CHOQUE/DANIEL RODRIGO M,</t>
+          <t>Departamento 5C - LUZ  TICONA QUISPE</t>
         </is>
       </c>
     </row>
@@ -2969,17 +3433,17 @@
         </is>
       </c>
       <c r="B179" s="4" t="n">
-        <v>186.57</v>
+        <v>179.21</v>
       </c>
       <c r="C179" s="5" t="n">
-        <v>186.57</v>
+        <v>179.21</v>
       </c>
     </row>
     <row r="180"/>
     <row r="181" ht="22" customHeight="1">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>Departamento 15E - WILMA IGLESIAS BEDOYA</t>
+          <t>Departamento 15B - MANUEL RAFAEL HIDALGO/STEFANY RAFAEL</t>
         </is>
       </c>
     </row>
@@ -2991,95 +3455,10 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>abr-25</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
-        <is>
-          <t>may-25</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="inlineStr">
-        <is>
-          <t>jun-25</t>
-        </is>
-      </c>
-      <c r="E182" s="2" t="inlineStr">
-        <is>
-          <t>jul-25</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr">
-        <is>
-          <t>ago-25</t>
-        </is>
-      </c>
-      <c r="G182" s="2" t="inlineStr">
-        <is>
-          <t>sep-25</t>
-        </is>
-      </c>
-      <c r="H182" s="2" t="inlineStr">
-        <is>
-          <t>oct-25</t>
-        </is>
-      </c>
-      <c r="I182" s="2" t="inlineStr">
-        <is>
-          <t>nov-25</t>
-        </is>
-      </c>
-      <c r="J182" s="2" t="inlineStr">
-        <is>
-          <t>dic-25</t>
-        </is>
-      </c>
-      <c r="K182" s="2" t="inlineStr">
-        <is>
-          <t>ene-26</t>
-        </is>
-      </c>
-      <c r="L182" s="2" t="inlineStr">
-        <is>
-          <t>feb-26</t>
-        </is>
-      </c>
-      <c r="M182" s="2" t="inlineStr">
-        <is>
-          <t>mar-26</t>
-        </is>
-      </c>
-      <c r="N182" s="2" t="inlineStr">
-        <is>
-          <t>abr-26</t>
-        </is>
-      </c>
-      <c r="O182" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="P182" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="Q182" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="R182" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="S182" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="T182" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3092,68 +3471,17 @@
         </is>
       </c>
       <c r="B183" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="C183" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="D183" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="E183" s="4" t="n">
-        <v>36</v>
-      </c>
-      <c r="F183" s="4" t="n">
-        <v>36.71</v>
-      </c>
-      <c r="G183" s="4" t="n">
-        <v>36.98</v>
-      </c>
-      <c r="H183" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="I183" s="4" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="J183" s="4" t="n">
-        <v>186.21</v>
-      </c>
-      <c r="K183" s="4" t="n">
-        <v>36.38</v>
-      </c>
-      <c r="L183" s="4" t="n">
-        <v>86.25</v>
-      </c>
-      <c r="M183" s="4" t="n">
-        <v>94.01000000000001</v>
-      </c>
-      <c r="N183" s="4" t="n">
-        <v>91</v>
-      </c>
-      <c r="O183" s="4" t="n">
-        <v>90.37</v>
-      </c>
-      <c r="P183" s="4" t="n">
-        <v>89.88</v>
-      </c>
-      <c r="Q183" s="4" t="n">
-        <v>50.91</v>
-      </c>
-      <c r="R183" s="4" t="n">
-        <v>241.35</v>
-      </c>
-      <c r="S183" s="4" t="n">
-        <v>242.02</v>
-      </c>
-      <c r="T183" s="5" t="n">
-        <v>1430.78</v>
+        <v>178.6</v>
+      </c>
+      <c r="C183" s="5" t="n">
+        <v>178.6</v>
       </c>
     </row>
     <row r="184"/>
     <row r="185" ht="22" customHeight="1">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>Departamento 15F - MICAELA DAFNE ALANES CUBA</t>
+          <t>Departamento 4C - SIRLEY VALENCIA/ANGEL VALENCVIA SIRPA</t>
         </is>
       </c>
     </row>
@@ -3165,15 +3493,10 @@
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>ago-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3186,20 +3509,17 @@
         </is>
       </c>
       <c r="B187" s="4" t="n">
-        <v>173.94</v>
-      </c>
-      <c r="C187" s="4" t="n">
-        <v>173.04</v>
-      </c>
-      <c r="D187" s="5" t="n">
-        <v>346.98</v>
+        <v>173.45</v>
+      </c>
+      <c r="C187" s="5" t="n">
+        <v>173.45</v>
       </c>
     </row>
     <row r="188"/>
     <row r="189" ht="22" customHeight="1">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>Departamento 16A - PABEL SAINZ E,/ERICK JARANDILLA</t>
+          <t>Departamento 7F - ROMAN CALDERON/ANGELA TERRAZAS M.</t>
         </is>
       </c>
     </row>
@@ -3211,20 +3531,10 @@
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>jul-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="D190" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3237,23 +3547,17 @@
         </is>
       </c>
       <c r="B191" s="4" t="n">
-        <v>180.63</v>
-      </c>
-      <c r="C191" s="4" t="n">
-        <v>177.85</v>
-      </c>
-      <c r="D191" s="4" t="n">
-        <v>173.14</v>
-      </c>
-      <c r="E191" s="5" t="n">
-        <v>531.62</v>
+        <v>168.73</v>
+      </c>
+      <c r="C191" s="5" t="n">
+        <v>168.73</v>
       </c>
     </row>
     <row r="192"/>
     <row r="193" ht="22" customHeight="1">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>Departamento 16F - ALVARO ANTICALLE</t>
+          <t>Departamento 10A - MARCELO USCAMAITA</t>
         </is>
       </c>
     </row>
@@ -3281,17 +3585,17 @@
         </is>
       </c>
       <c r="B195" s="4" t="n">
-        <v>192.48</v>
+        <v>166.29</v>
       </c>
       <c r="C195" s="5" t="n">
-        <v>192.48</v>
+        <v>166.29</v>
       </c>
     </row>
     <row r="196"/>
     <row r="197" ht="22" customHeight="1">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>Departamento 18C - SANDRA MALLEA</t>
+          <t>Departamento 20C - CATHERIN ROJAS C,/MIGUELA,CORONADO</t>
         </is>
       </c>
     </row>
@@ -3303,90 +3607,10 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>may-25</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
-        <is>
-          <t>jun-25</t>
-        </is>
-      </c>
-      <c r="D198" s="2" t="inlineStr">
-        <is>
-          <t>jul-25</t>
-        </is>
-      </c>
-      <c r="E198" s="2" t="inlineStr">
-        <is>
-          <t>ago-25</t>
-        </is>
-      </c>
-      <c r="F198" s="2" t="inlineStr">
-        <is>
-          <t>sep-25</t>
-        </is>
-      </c>
-      <c r="G198" s="2" t="inlineStr">
-        <is>
-          <t>oct-25</t>
-        </is>
-      </c>
-      <c r="H198" s="2" t="inlineStr">
-        <is>
-          <t>nov-25</t>
-        </is>
-      </c>
-      <c r="I198" s="2" t="inlineStr">
-        <is>
-          <t>dic-25</t>
-        </is>
-      </c>
-      <c r="J198" s="2" t="inlineStr">
-        <is>
-          <t>ene-26</t>
-        </is>
-      </c>
-      <c r="K198" s="2" t="inlineStr">
-        <is>
-          <t>feb-26</t>
-        </is>
-      </c>
-      <c r="L198" s="2" t="inlineStr">
-        <is>
-          <t>mar-26</t>
-        </is>
-      </c>
-      <c r="M198" s="2" t="inlineStr">
-        <is>
-          <t>abr-26</t>
-        </is>
-      </c>
-      <c r="N198" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="O198" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="P198" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="Q198" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="R198" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="S198" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3399,65 +3623,17 @@
         </is>
       </c>
       <c r="B199" s="4" t="n">
-        <v>116</v>
-      </c>
-      <c r="C199" s="4" t="n">
-        <v>117</v>
-      </c>
-      <c r="D199" s="4" t="n">
-        <v>115</v>
-      </c>
-      <c r="E199" s="4" t="n">
-        <v>114.11</v>
-      </c>
-      <c r="F199" s="4" t="n">
-        <v>114.08</v>
-      </c>
-      <c r="G199" s="4" t="n">
-        <v>114.17</v>
-      </c>
-      <c r="H199" s="4" t="n">
-        <v>114.21</v>
-      </c>
-      <c r="I199" s="4" t="n">
-        <v>114</v>
-      </c>
-      <c r="J199" s="4" t="n">
-        <v>114</v>
-      </c>
-      <c r="K199" s="4" t="n">
-        <v>145.3</v>
-      </c>
-      <c r="L199" s="4" t="n">
-        <v>145.04</v>
-      </c>
-      <c r="M199" s="4" t="n">
-        <v>145.37</v>
-      </c>
-      <c r="N199" s="4" t="n">
-        <v>145.46</v>
-      </c>
-      <c r="O199" s="4" t="n">
-        <v>145.23</v>
-      </c>
-      <c r="P199" s="4" t="n">
-        <v>145.29</v>
-      </c>
-      <c r="Q199" s="4" t="n">
-        <v>145.33</v>
-      </c>
-      <c r="R199" s="4" t="n">
-        <v>146.57</v>
-      </c>
-      <c r="S199" s="5" t="n">
-        <v>2196.16</v>
+        <v>145</v>
+      </c>
+      <c r="C199" s="5" t="n">
+        <v>145</v>
       </c>
     </row>
     <row r="200"/>
     <row r="201" ht="22" customHeight="1">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>Departamento 18DE - SANDRO MEDRANO</t>
+          <t>Departamento 21B - ROLY CHAVEZ HUANCA</t>
         </is>
       </c>
     </row>
@@ -3469,30 +3645,10 @@
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>may-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="D202" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="E202" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="F202" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="G202" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3505,29 +3661,17 @@
         </is>
       </c>
       <c r="B203" s="4" t="n">
-        <v>69</v>
-      </c>
-      <c r="C203" s="4" t="n">
-        <v>38.66</v>
-      </c>
-      <c r="D203" s="4" t="n">
-        <v>69</v>
-      </c>
-      <c r="E203" s="4" t="n">
-        <v>69</v>
-      </c>
-      <c r="F203" s="4" t="n">
-        <v>69</v>
-      </c>
-      <c r="G203" s="5" t="n">
-        <v>314.66</v>
+        <v>143.83</v>
+      </c>
+      <c r="C203" s="5" t="n">
+        <v>143.83</v>
       </c>
     </row>
     <row r="204"/>
     <row r="205" ht="22" customHeight="1">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>Departamento 20B - RAQUEL GUTIERREZ FLORES</t>
+          <t>Departamento &lt;NA&gt;AC - LAVANDERIA</t>
         </is>
       </c>
     </row>
@@ -3565,23 +3709,23 @@
         </is>
       </c>
       <c r="B207" s="4" t="n">
-        <v>228.7</v>
+        <v>46.16</v>
       </c>
       <c r="C207" s="4" t="n">
-        <v>231.79</v>
+        <v>45.07</v>
       </c>
       <c r="D207" s="4" t="n">
-        <v>226.48</v>
+        <v>45.68</v>
       </c>
       <c r="E207" s="5" t="n">
-        <v>686.97</v>
+        <v>136.91</v>
       </c>
     </row>
     <row r="208"/>
     <row r="209" ht="22" customHeight="1">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>Departamento 20C - CATHERIN ROJAS C,/MIGUELA,CORONADO</t>
+          <t>Departamento 11D - LAURA GEMIO/WILMER CABRERA G.</t>
         </is>
       </c>
     </row>
@@ -3609,17 +3753,17 @@
         </is>
       </c>
       <c r="B211" s="4" t="n">
-        <v>145</v>
+        <v>132.18</v>
       </c>
       <c r="C211" s="5" t="n">
-        <v>145</v>
+        <v>132.18</v>
       </c>
     </row>
     <row r="212"/>
     <row r="213" ht="22" customHeight="1">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>Departamento 20DE - GRACE FERNANDEZ</t>
+          <t>Departamento 5D - MARCELO LOZA/ MARCOS RODRIGUEZ</t>
         </is>
       </c>
     </row>
@@ -3631,45 +3775,10 @@
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>feb-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
-        <is>
-          <t>mar-26</t>
-        </is>
-      </c>
-      <c r="D214" s="2" t="inlineStr">
-        <is>
-          <t>abr-26</t>
-        </is>
-      </c>
-      <c r="E214" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="F214" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="G214" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="H214" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="I214" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="J214" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3682,38 +3791,17 @@
         </is>
       </c>
       <c r="B215" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="C215" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="D215" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="E215" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="F215" s="4" t="n">
-        <v>70.03</v>
-      </c>
-      <c r="G215" s="4" t="n">
-        <v>69.97</v>
-      </c>
-      <c r="H215" s="4" t="n">
-        <v>69.97</v>
-      </c>
-      <c r="I215" s="4" t="n">
-        <v>69.95999999999999</v>
-      </c>
-      <c r="J215" s="5" t="n">
-        <v>559.9300000000001</v>
+        <v>125.2</v>
+      </c>
+      <c r="C215" s="5" t="n">
+        <v>125.2</v>
       </c>
     </row>
     <row r="216"/>
     <row r="217" ht="22" customHeight="1">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>Departamento 21B - ROLY CHAVEZ HUANCA</t>
+          <t>Departamento 12D - ERIKA LEON HERBAS</t>
         </is>
       </c>
     </row>
@@ -3741,17 +3829,17 @@
         </is>
       </c>
       <c r="B219" s="4" t="n">
-        <v>143.83</v>
+        <v>106.54</v>
       </c>
       <c r="C219" s="5" t="n">
-        <v>143.83</v>
+        <v>106.54</v>
       </c>
     </row>
     <row r="220"/>
     <row r="221" ht="22" customHeight="1">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>Departamento 22B - FABIOLA LAURA VARGAS</t>
+          <t>Departamento 7D - MARTHA LIZARAZU/FROILAN LOPEZ CH.</t>
         </is>
       </c>
     </row>
@@ -3763,60 +3851,10 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>nov-25</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
-        <is>
-          <t>dic-25</t>
-        </is>
-      </c>
-      <c r="D222" s="2" t="inlineStr">
-        <is>
-          <t>ene-26</t>
-        </is>
-      </c>
-      <c r="E222" s="2" t="inlineStr">
-        <is>
-          <t>feb-26</t>
-        </is>
-      </c>
-      <c r="F222" s="2" t="inlineStr">
-        <is>
-          <t>mar-26</t>
-        </is>
-      </c>
-      <c r="G222" s="2" t="inlineStr">
-        <is>
-          <t>abr-26</t>
-        </is>
-      </c>
-      <c r="H222" s="2" t="inlineStr">
-        <is>
-          <t>may-26</t>
-        </is>
-      </c>
-      <c r="I222" s="2" t="inlineStr">
-        <is>
-          <t>jun-26</t>
-        </is>
-      </c>
-      <c r="J222" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="K222" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="L222" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="M222" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3829,47 +3867,17 @@
         </is>
       </c>
       <c r="B223" s="4" t="n">
-        <v>292.3</v>
-      </c>
-      <c r="C223" s="4" t="n">
-        <v>263.15</v>
-      </c>
-      <c r="D223" s="4" t="n">
-        <v>282.93</v>
-      </c>
-      <c r="E223" s="4" t="n">
-        <v>317.65</v>
-      </c>
-      <c r="F223" s="4" t="n">
-        <v>317.78</v>
-      </c>
-      <c r="G223" s="4" t="n">
-        <v>336.63</v>
-      </c>
-      <c r="H223" s="4" t="n">
-        <v>317</v>
-      </c>
-      <c r="I223" s="4" t="n">
-        <v>317</v>
-      </c>
-      <c r="J223" s="4" t="n">
-        <v>317</v>
-      </c>
-      <c r="K223" s="4" t="n">
-        <v>317</v>
-      </c>
-      <c r="L223" s="4" t="n">
-        <v>342.22</v>
-      </c>
-      <c r="M223" s="5" t="n">
-        <v>3420.66</v>
+        <v>92.09999999999999</v>
+      </c>
+      <c r="C223" s="5" t="n">
+        <v>92.09999999999999</v>
       </c>
     </row>
     <row r="224"/>
     <row r="225" ht="22" customHeight="1">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>Departamento &lt;NA&gt;AC - LAVANDERIA</t>
+          <t>Departamento &lt;NA&gt;nan - GIMNASIO</t>
         </is>
       </c>
     </row>
@@ -3907,23 +3915,23 @@
         </is>
       </c>
       <c r="B227" s="4" t="n">
-        <v>46.16</v>
+        <v>0.48</v>
       </c>
       <c r="C227" s="4" t="n">
-        <v>45.07</v>
+        <v>0.05</v>
       </c>
       <c r="D227" s="4" t="n">
-        <v>45.68</v>
+        <v>0.59</v>
       </c>
       <c r="E227" s="5" t="n">
-        <v>136.91</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="228"/>
     <row r="229" ht="22" customHeight="1">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>Departamento &lt;NA&gt;nan - GIMNASIO</t>
+          <t>Departamento 13D - MARIA LUISA PEÑALOZA VILA</t>
         </is>
       </c>
     </row>
@@ -3935,20 +3943,15 @@
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>jul-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>ago-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="E230" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3961,78 +3964,75 @@
         </is>
       </c>
       <c r="B231" s="4" t="n">
-        <v>0.48</v>
+        <v>0.01</v>
       </c>
       <c r="C231" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="D231" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E231" s="5" t="n">
-        <v>1.12</v>
+      <c r="D231" s="5" t="n">
+        <v>0.06</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="58">
+    <mergeCell ref="A137:C137"/>
+    <mergeCell ref="A77:E77"/>
     <mergeCell ref="A177:C177"/>
+    <mergeCell ref="A221:C221"/>
     <mergeCell ref="A193:C193"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A133:C133"/>
     <mergeCell ref="A217:C217"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A53:G53"/>
-    <mergeCell ref="A89:C89"/>
+    <mergeCell ref="A17:S17"/>
+    <mergeCell ref="A109:D109"/>
+    <mergeCell ref="A145:C145"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A149:C149"/>
+    <mergeCell ref="A101:C101"/>
+    <mergeCell ref="A189:C189"/>
     <mergeCell ref="A225:E225"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A101:C101"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A105:C105"/>
-    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="A81:G81"/>
+    <mergeCell ref="A93:D93"/>
+    <mergeCell ref="A113:C113"/>
+    <mergeCell ref="A117:G117"/>
     <mergeCell ref="A129:C129"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A85:F85"/>
+    <mergeCell ref="A213:C213"/>
+    <mergeCell ref="A229:D229"/>
+    <mergeCell ref="A185:C185"/>
     <mergeCell ref="A205:E205"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A157:D157"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A201:G201"/>
-    <mergeCell ref="A5:R5"/>
-    <mergeCell ref="A141:O141"/>
-    <mergeCell ref="A109:C109"/>
-    <mergeCell ref="A49:G49"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A81:C81"/>
+    <mergeCell ref="A141:C141"/>
+    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="A181:C181"/>
+    <mergeCell ref="A41:H41"/>
     <mergeCell ref="A125:C125"/>
-    <mergeCell ref="A149:H149"/>
-    <mergeCell ref="A189:E189"/>
     <mergeCell ref="A209:C209"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A93:F93"/>
-    <mergeCell ref="A117:C117"/>
-    <mergeCell ref="A197:S197"/>
+    <mergeCell ref="A49:J49"/>
+    <mergeCell ref="A121:C121"/>
+    <mergeCell ref="A161:C161"/>
+    <mergeCell ref="A165:C165"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A13:O13"/>
+    <mergeCell ref="A9:F9"/>
     <mergeCell ref="A173:C173"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A77:C77"/>
-    <mergeCell ref="A137:D137"/>
-    <mergeCell ref="A73:C73"/>
-    <mergeCell ref="A41:J41"/>
-    <mergeCell ref="A221:M221"/>
-    <mergeCell ref="A181:T181"/>
-    <mergeCell ref="A97:K97"/>
-    <mergeCell ref="A133:J133"/>
+    <mergeCell ref="A69:J69"/>
+    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A65:J65"/>
+    <mergeCell ref="A33:T33"/>
+    <mergeCell ref="A157:C157"/>
+    <mergeCell ref="A201:C201"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A53:E53"/>
     <mergeCell ref="A169:C169"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="A145:D145"/>
-    <mergeCell ref="A165:E165"/>
-    <mergeCell ref="A161:E161"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="A121:K121"/>
+    <mergeCell ref="A89:D89"/>
+    <mergeCell ref="A105:D105"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A197:C197"/>
+    <mergeCell ref="A61:F61"/>
     <mergeCell ref="A153:C153"/>
-    <mergeCell ref="A113:D113"/>
-    <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="A213:J213"/>
-    <mergeCell ref="A229:E229"/>
-    <mergeCell ref="A185:D185"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Actualizacion cuadro de mora
</commit_message>
<xml_diff>
--- a/Edificio Miraflores/reporte_mora_miraflores.xlsx
+++ b/Edificio Miraflores/reporte_mora_miraflores.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T231"/>
+  <dimension ref="A1:T223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -520,7 +520,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>sep-25</t>
+          <t>sept-25</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>sep-25</t>
+          <t>sept-25</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>sep-25</t>
+          <t>sept-25</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ges_ant</t>
+          <t>gestiones anteriores</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>sep-25</t>
+          <t>sept-25</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3671,7 +3671,7 @@
     <row r="205" ht="22" customHeight="1">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>Departamento &lt;NA&gt;AC - LAVANDERIA</t>
+          <t>Departamento 11D - LAURA GEMIO/WILMER CABRERA G.</t>
         </is>
       </c>
     </row>
@@ -3683,20 +3683,10 @@
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>jul-26</t>
+          <t>sep-26</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="D206" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="E206" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3709,23 +3699,17 @@
         </is>
       </c>
       <c r="B207" s="4" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="C207" s="4" t="n">
-        <v>45.07</v>
-      </c>
-      <c r="D207" s="4" t="n">
-        <v>45.68</v>
-      </c>
-      <c r="E207" s="5" t="n">
-        <v>136.91</v>
+        <v>132.18</v>
+      </c>
+      <c r="C207" s="5" t="n">
+        <v>132.18</v>
       </c>
     </row>
     <row r="208"/>
     <row r="209" ht="22" customHeight="1">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>Departamento 11D - LAURA GEMIO/WILMER CABRERA G.</t>
+          <t>Departamento 5D - MARCELO LOZA/ MARCOS RODRIGUEZ</t>
         </is>
       </c>
     </row>
@@ -3753,17 +3737,17 @@
         </is>
       </c>
       <c r="B211" s="4" t="n">
-        <v>132.18</v>
+        <v>125.2</v>
       </c>
       <c r="C211" s="5" t="n">
-        <v>132.18</v>
+        <v>125.2</v>
       </c>
     </row>
     <row r="212"/>
     <row r="213" ht="22" customHeight="1">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>Departamento 5D - MARCELO LOZA/ MARCOS RODRIGUEZ</t>
+          <t>Departamento 12D - ERIKA LEON HERBAS</t>
         </is>
       </c>
     </row>
@@ -3791,17 +3775,17 @@
         </is>
       </c>
       <c r="B215" s="4" t="n">
-        <v>125.2</v>
+        <v>106.54</v>
       </c>
       <c r="C215" s="5" t="n">
-        <v>125.2</v>
+        <v>106.54</v>
       </c>
     </row>
     <row r="216"/>
     <row r="217" ht="22" customHeight="1">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>Departamento 12D - ERIKA LEON HERBAS</t>
+          <t>Departamento 7D - MARTHA LIZARAZU/FROILAN LOPEZ CH.</t>
         </is>
       </c>
     </row>
@@ -3829,17 +3813,17 @@
         </is>
       </c>
       <c r="B219" s="4" t="n">
-        <v>106.54</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C219" s="5" t="n">
-        <v>106.54</v>
+        <v>92.09999999999999</v>
       </c>
     </row>
     <row r="220"/>
     <row r="221" ht="22" customHeight="1">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>Departamento 7D - MARTHA LIZARAZU/FROILAN LOPEZ CH.</t>
+          <t>Departamento 13D - MARIA LUISA PEÑALOZA VILA</t>
         </is>
       </c>
     </row>
@@ -3851,10 +3835,15 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>sep-26</t>
+          <t>ago-26</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>sep-26</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3867,118 +3856,20 @@
         </is>
       </c>
       <c r="B223" s="4" t="n">
-        <v>92.09999999999999</v>
-      </c>
-      <c r="C223" s="5" t="n">
-        <v>92.09999999999999</v>
-      </c>
-    </row>
-    <row r="224"/>
-    <row r="225" ht="22" customHeight="1">
-      <c r="A225" s="1" t="inlineStr">
-        <is>
-          <t>Departamento &lt;NA&gt;nan - GIMNASIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" s="2" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B226" s="2" t="inlineStr">
-        <is>
-          <t>jul-26</t>
-        </is>
-      </c>
-      <c r="C226" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="D226" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="E226" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" s="3" t="inlineStr">
-        <is>
-          <t>Expensas</t>
-        </is>
-      </c>
-      <c r="B227" s="4" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="C227" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C223" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="D227" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E227" s="5" t="n">
-        <v>1.12</v>
-      </c>
-    </row>
-    <row r="228"/>
-    <row r="229" ht="22" customHeight="1">
-      <c r="A229" s="1" t="inlineStr">
-        <is>
-          <t>Departamento 13D - MARIA LUISA PEÑALOZA VILA</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" s="2" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B230" s="2" t="inlineStr">
-        <is>
-          <t>ago-26</t>
-        </is>
-      </c>
-      <c r="C230" s="2" t="inlineStr">
-        <is>
-          <t>sep-26</t>
-        </is>
-      </c>
-      <c r="D230" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" s="3" t="inlineStr">
-        <is>
-          <t>Expensas</t>
-        </is>
-      </c>
-      <c r="B231" s="4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C231" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D231" s="5" t="n">
+      <c r="D223" s="5" t="n">
         <v>0.06</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="58">
+  <mergeCells count="56">
     <mergeCell ref="A137:C137"/>
     <mergeCell ref="A77:E77"/>
     <mergeCell ref="A177:C177"/>
-    <mergeCell ref="A221:C221"/>
     <mergeCell ref="A193:C193"/>
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="A73:E73"/>
@@ -3992,16 +3883,13 @@
     <mergeCell ref="A149:C149"/>
     <mergeCell ref="A101:C101"/>
     <mergeCell ref="A189:C189"/>
-    <mergeCell ref="A225:E225"/>
     <mergeCell ref="A81:G81"/>
     <mergeCell ref="A93:D93"/>
     <mergeCell ref="A113:C113"/>
     <mergeCell ref="A117:G117"/>
     <mergeCell ref="A129:C129"/>
     <mergeCell ref="A213:C213"/>
-    <mergeCell ref="A229:D229"/>
     <mergeCell ref="A185:C185"/>
-    <mergeCell ref="A205:E205"/>
     <mergeCell ref="A141:C141"/>
     <mergeCell ref="A25:K25"/>
     <mergeCell ref="A181:C181"/>
@@ -4021,6 +3909,7 @@
     <mergeCell ref="A85:E85"/>
     <mergeCell ref="A65:J65"/>
     <mergeCell ref="A33:T33"/>
+    <mergeCell ref="A221:D221"/>
     <mergeCell ref="A157:C157"/>
     <mergeCell ref="A201:C201"/>
     <mergeCell ref="A37:G37"/>
@@ -4033,6 +3922,7 @@
     <mergeCell ref="A61:F61"/>
     <mergeCell ref="A153:C153"/>
     <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A205:C205"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>